<commit_message>
fix: D30 label shows BOL/EOL per ageing_type + update Sizing_template.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Sizing_template.xlsx
+++ b/templates/Sizing_template.xlsx
@@ -354,7 +354,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -571,115 +571,115 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="7" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="9" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="7" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -724,7 +724,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{82EE31AC-07DB-40B3-A13F-4C4C308D6B25}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82EE31AC-07DB-40B3-A13F-4C4C308D6B25}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -774,7 +774,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{72F9E248-A0A2-45EF-827F-2EB33A67B7D6}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72F9E248-A0A2-45EF-827F-2EB33A67B7D6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1139,67 +1139,67 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:15" ht="80.099999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="25"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="46"/>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="39.950000000000003" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="27"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="48"/>
       <c r="H3" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="32"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="53"/>
     </row>
     <row r="5" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
+      <c r="B5" s="55"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="58"/>
     </row>
     <row r="6" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
     </row>
     <row r="7" spans="1:15" ht="54" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
@@ -1240,376 +1240,376 @@
       <c r="H8" s="8"/>
     </row>
     <row r="9" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
+      <c r="A9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
     </row>
     <row r="10" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="42" t="s">
+      <c r="A10" s="24"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="44"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="36"/>
     </row>
     <row r="11" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="40"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
       <c r="D11" s="21"/>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="44"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="36"/>
     </row>
     <row r="12" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
       <c r="D12" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="45"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="47"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="39"/>
     </row>
     <row r="13" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
       <c r="D13" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
-      <c r="J13" s="59"/>
-      <c r="K13" s="59"/>
-      <c r="L13" s="59"/>
-      <c r="M13" s="59"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="36"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
     </row>
     <row r="14" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="39" t="s">
+      <c r="A14" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
       <c r="D14" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="42"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="44"/>
-      <c r="J14" s="59"/>
-      <c r="K14" s="59"/>
-      <c r="L14" s="59"/>
-      <c r="M14" s="59"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="36"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="23"/>
       <c r="O14" s="9"/>
     </row>
     <row r="15" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
       <c r="D15" s="21"/>
-      <c r="E15" s="42" t="s">
+      <c r="E15" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="44"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="59"/>
-      <c r="M15" s="59"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="36"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="23"/>
     </row>
     <row r="16" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="39" t="s">
+      <c r="A16" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
       <c r="D16" s="21"/>
-      <c r="E16" s="42" t="s">
+      <c r="E16" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="44"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="59"/>
-      <c r="L16" s="59"/>
-      <c r="M16" s="59"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="36"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
     </row>
     <row r="17" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
       <c r="D17" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="45"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="47"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="59"/>
-      <c r="L17" s="59"/>
-      <c r="M17" s="59"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="39"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
     </row>
     <row r="18" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="39" t="s">
+      <c r="A18" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
       <c r="D18" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="45"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="47"/>
-      <c r="J18" s="59"/>
-      <c r="K18" s="59"/>
-      <c r="L18" s="59"/>
-      <c r="M18" s="59"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="39"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+      <c r="M18" s="23"/>
       <c r="N18" s="17"/>
     </row>
     <row r="19" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="39" t="s">
+      <c r="A19" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
       <c r="D19" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="54"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="56"/>
-      <c r="J19" s="59"/>
-      <c r="K19" s="59"/>
-      <c r="L19" s="59"/>
-      <c r="M19" s="59"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="30"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
       <c r="N19" s="17"/>
     </row>
     <row r="20" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
       <c r="D20" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E20" s="54"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="56"/>
-      <c r="J20" s="59"/>
-      <c r="K20" s="59"/>
-      <c r="L20" s="59"/>
-      <c r="M20" s="59"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="30"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="23"/>
       <c r="N20" s="17"/>
     </row>
     <row r="21" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="39" t="s">
+      <c r="A21" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
       <c r="D21" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E21" s="54"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="56"/>
-      <c r="J21" s="59"/>
-      <c r="K21" s="59"/>
-      <c r="L21" s="59"/>
-      <c r="M21" s="59"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="30"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="39" t="s">
+      <c r="A22" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
       <c r="D22" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="54"/>
-      <c r="F22" s="55"/>
-      <c r="G22" s="55"/>
-      <c r="H22" s="56"/>
-      <c r="J22" s="59"/>
-      <c r="K22" s="59"/>
-      <c r="L22" s="59"/>
-      <c r="M22" s="59"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="30"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
     </row>
     <row r="23" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="57" t="s">
+      <c r="A23" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="58"/>
-      <c r="C23" s="58"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
       <c r="D23" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E23" s="45"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="47"/>
-      <c r="J23" s="59"/>
-      <c r="K23" s="59"/>
-      <c r="L23" s="59"/>
-      <c r="M23" s="59"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="39"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="23"/>
     </row>
     <row r="24" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="57" t="s">
+      <c r="A24" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="58"/>
-      <c r="C24" s="58"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
       <c r="D24" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E24" s="45"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="47"/>
-      <c r="J24" s="59"/>
-      <c r="K24" s="59"/>
-      <c r="L24" s="59"/>
-      <c r="M24" s="59"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="39"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="23"/>
     </row>
     <row r="25" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="57" t="s">
+      <c r="A25" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="58"/>
-      <c r="C25" s="58"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
       <c r="D25" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E25" s="45"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="47"/>
-      <c r="J25" s="59"/>
-      <c r="K25" s="59"/>
-      <c r="L25" s="59"/>
-      <c r="M25" s="59"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="39"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
     </row>
     <row r="26" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="58"/>
-      <c r="C26" s="58"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
       <c r="D26" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="45"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="46"/>
-      <c r="H26" s="47"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="59"/>
-      <c r="L26" s="59"/>
-      <c r="M26" s="59"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="39"/>
+      <c r="J26" s="23"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
     </row>
     <row r="27" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="39" t="s">
+      <c r="A27" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="40"/>
-      <c r="C27" s="40"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
       <c r="D27" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E27" s="42"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
-      <c r="J27" s="59"/>
-      <c r="K27" s="59"/>
-      <c r="L27" s="59"/>
-      <c r="M27" s="59"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="36"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
     </row>
     <row r="28" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="40"/>
-      <c r="C28" s="40"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
       <c r="D28" s="21"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="50"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="51"/>
-      <c r="J28" s="59"/>
-      <c r="K28" s="59"/>
-      <c r="L28" s="59"/>
-      <c r="M28" s="59"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="33"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
     </row>
     <row r="29" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="39" t="s">
+      <c r="A29" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="40"/>
-      <c r="C29" s="40"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
       <c r="D29" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="42"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="44"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="36"/>
       <c r="J29" s="19"/>
       <c r="K29" s="20"/>
       <c r="L29" s="18"/>
     </row>
     <row r="30" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="57" t="s">
+      <c r="A30" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="58"/>
-      <c r="C30" s="58"/>
-      <c r="D30" s="23" t="s">
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="E30" s="49"/>
-      <c r="F30" s="50"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="51"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="33"/>
     </row>
     <row r="31" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
@@ -1632,56 +1632,56 @@
       <c r="H32" s="13"/>
     </row>
     <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B33" s="52"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="52"/>
-      <c r="H33" s="52"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="41"/>
+      <c r="H33" s="41"/>
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="52"/>
-      <c r="B34" s="52"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
+      <c r="A34" s="41"/>
+      <c r="B34" s="41"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="41"/>
+      <c r="G34" s="41"/>
+      <c r="H34" s="41"/>
     </row>
     <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="52"/>
-      <c r="B35" s="52"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="52"/>
-      <c r="H35" s="52"/>
+      <c r="A35" s="41"/>
+      <c r="B35" s="41"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="41"/>
+      <c r="G35" s="41"/>
+      <c r="H35" s="41"/>
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
-      <c r="B36" s="52"/>
-      <c r="C36" s="52"/>
-      <c r="D36" s="52"/>
-      <c r="E36" s="52"/>
-      <c r="F36" s="52"/>
-      <c r="G36" s="52"/>
-      <c r="H36" s="52"/>
+      <c r="A36" s="41"/>
+      <c r="B36" s="41"/>
+      <c r="C36" s="41"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="41"/>
+      <c r="H36" s="41"/>
     </row>
     <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
-      <c r="B37" s="52"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="52"/>
-      <c r="H37" s="52"/>
+      <c r="A37" s="41"/>
+      <c r="B37" s="41"/>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="41"/>
+      <c r="G37" s="41"/>
+      <c r="H37" s="41"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="14"/>
@@ -1691,33 +1691,58 @@
       <c r="H48" s="15"/>
     </row>
     <row r="49" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="53" t="s">
+      <c r="A49" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="B49" s="53"/>
-      <c r="C49" s="53"/>
-      <c r="D49" s="53"/>
+      <c r="B49" s="42"/>
+      <c r="C49" s="42"/>
+      <c r="D49" s="42"/>
       <c r="F49" s="16"/>
       <c r="G49" s="16"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="48" t="s">
+      <c r="A50" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="48"/>
-      <c r="C50" s="48"/>
-      <c r="D50" s="48"/>
+      <c r="B50" s="40"/>
+      <c r="C50" s="40"/>
+      <c r="D50" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="E23:H23"/>
+    <mergeCell ref="E18:H18"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="E14:H14"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="E29:H29"/>
+    <mergeCell ref="E30:H30"/>
+    <mergeCell ref="A33:H37"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="E28:H28"/>
+    <mergeCell ref="E27:H27"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="E25:H25"/>
+    <mergeCell ref="E26:H26"/>
     <mergeCell ref="E19:H19"/>
     <mergeCell ref="E20:H20"/>
     <mergeCell ref="E21:H21"/>
@@ -1727,42 +1752,17 @@
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A19:C19"/>
-    <mergeCell ref="E28:H28"/>
-    <mergeCell ref="E27:H27"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="E25:H25"/>
-    <mergeCell ref="E26:H26"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="E29:H29"/>
-    <mergeCell ref="E30:H30"/>
-    <mergeCell ref="A33:H37"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="E12:H12"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="E14:H14"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A14:C14"/>
     <mergeCell ref="E15:H15"/>
     <mergeCell ref="E16:H16"/>
     <mergeCell ref="E17:H17"/>
-    <mergeCell ref="E23:H23"/>
-    <mergeCell ref="E18:H18"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="E10:H10"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A49" r:id="rId1"/>

</xml_diff>